<commit_message>
Corrections and pipelines/db changes
</commit_message>
<xml_diff>
--- a/clinical_tables/clinical_CHIKV.xlsx
+++ b/clinical_tables/clinical_CHIKV.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="65">
   <si>
     <t>Category</t>
   </si>
@@ -66,22 +66,19 @@
     <t>15-19</t>
   </si>
   <si>
-    <t>20-29</t>
-  </si>
-  <si>
-    <t>30-39</t>
-  </si>
-  <si>
-    <t>40-49</t>
+    <t>20-39</t>
+  </si>
+  <si>
+    <t>40-59</t>
   </si>
   <si>
     <t>5-9</t>
   </si>
   <si>
-    <t>50-59</t>
-  </si>
-  <si>
-    <t>60-69</t>
+    <t>60-64</t>
+  </si>
+  <si>
+    <t>65-69</t>
   </si>
   <si>
     <t>70-79</t>
@@ -99,22 +96,13 @@
     <t>Chikungunya</t>
   </si>
   <si>
-    <t>Dengue</t>
-  </si>
-  <si>
-    <t>Dengue c/ complicacoes (antigo)</t>
-  </si>
-  <si>
-    <t>Dengue classico (schema antigo)</t>
-  </si>
-  <si>
-    <t>Descartado</t>
-  </si>
-  <si>
     <t>Inconclusivo</t>
   </si>
   <si>
     <t>codigo_0</t>
+  </si>
+  <si>
+    <t>codigo_10</t>
   </si>
   <si>
     <t>Clinico-epidemiologico</t>
@@ -568,7 +556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1">
@@ -614,37 +602,37 @@
         <v>12</v>
       </c>
       <c r="B2">
-        <v>7253</v>
+        <v>4842</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>3235</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>1501</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>1949</v>
       </c>
       <c r="F2">
-        <v>0</v>
+        <v>1178</v>
       </c>
       <c r="G2">
-        <v>3328</v>
+        <v>1979</v>
       </c>
       <c r="H2">
-        <v>6927</v>
+        <v>3665</v>
       </c>
       <c r="I2">
-        <v>5982</v>
+        <v>2858</v>
       </c>
       <c r="J2">
-        <v>9313</v>
+        <v>4650</v>
       </c>
       <c r="K2">
-        <v>6963</v>
+        <v>2643</v>
       </c>
       <c r="L2">
-        <v>3878</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -652,37 +640,37 @@
         <v>13</v>
       </c>
       <c r="B3">
-        <v>16983</v>
+        <v>12440</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>10373</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>4372</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>6089</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>3410</v>
       </c>
       <c r="G3">
-        <v>6433</v>
+        <v>4188</v>
       </c>
       <c r="H3">
-        <v>15183</v>
+        <v>9194</v>
       </c>
       <c r="I3">
-        <v>15219</v>
+        <v>8307</v>
       </c>
       <c r="J3">
-        <v>23443</v>
+        <v>13067</v>
       </c>
       <c r="K3">
-        <v>15114</v>
+        <v>7074</v>
       </c>
       <c r="L3">
-        <v>8843</v>
+        <v>3995</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -690,37 +678,37 @@
         <v>14</v>
       </c>
       <c r="B4">
-        <v>21359</v>
+        <v>15795</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>14047</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>5950</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>7999</v>
       </c>
       <c r="F4">
-        <v>0</v>
+        <v>3892</v>
       </c>
       <c r="G4">
-        <v>7189</v>
+        <v>4678</v>
       </c>
       <c r="H4">
-        <v>16928</v>
+        <v>10105</v>
       </c>
       <c r="I4">
-        <v>18309</v>
+        <v>9719</v>
       </c>
       <c r="J4">
-        <v>28962</v>
+        <v>15867</v>
       </c>
       <c r="K4">
-        <v>18206</v>
+        <v>8118</v>
       </c>
       <c r="L4">
-        <v>10744</v>
+        <v>4641</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -728,37 +716,37 @@
         <v>15</v>
       </c>
       <c r="B5">
-        <v>52688</v>
+        <v>81175</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>69039</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>30008</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>44522</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>25923</v>
       </c>
       <c r="G5">
-        <v>21268</v>
+        <v>29794</v>
       </c>
       <c r="H5">
-        <v>47622</v>
+        <v>60555</v>
       </c>
       <c r="I5">
-        <v>47066</v>
+        <v>52097</v>
       </c>
       <c r="J5">
-        <v>70859</v>
+        <v>80714</v>
       </c>
       <c r="K5">
-        <v>43882</v>
+        <v>40899</v>
       </c>
       <c r="L5">
-        <v>24334</v>
+        <v>21604</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -766,37 +754,37 @@
         <v>16</v>
       </c>
       <c r="B6">
-        <v>57053</v>
+        <v>71100</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>53437</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>27737</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>42022</v>
       </c>
       <c r="F6">
-        <v>0</v>
+        <v>24668</v>
       </c>
       <c r="G6">
-        <v>23809</v>
+        <v>28437</v>
       </c>
       <c r="H6">
-        <v>49547</v>
+        <v>55147</v>
       </c>
       <c r="I6">
-        <v>45366</v>
+        <v>49600</v>
       </c>
       <c r="J6">
-        <v>67582</v>
+        <v>84630</v>
       </c>
       <c r="K6">
-        <v>42904</v>
+        <v>39245</v>
       </c>
       <c r="L6">
-        <v>21145</v>
+        <v>20252</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -804,37 +792,37 @@
         <v>17</v>
       </c>
       <c r="B7">
-        <v>50523</v>
+        <v>8946</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>7159</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>2934</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>4245</v>
       </c>
       <c r="F7">
-        <v>0</v>
+        <v>2651</v>
       </c>
       <c r="G7">
-        <v>22657</v>
+        <v>3626</v>
       </c>
       <c r="H7">
-        <v>46684</v>
+        <v>7036</v>
       </c>
       <c r="I7">
-        <v>44775</v>
+        <v>5911</v>
       </c>
       <c r="J7">
-        <v>71047</v>
+        <v>9786</v>
       </c>
       <c r="K7">
-        <v>41228</v>
+        <v>5345</v>
       </c>
       <c r="L7">
-        <v>20000</v>
+        <v>2867</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -842,37 +830,37 @@
         <v>18</v>
       </c>
       <c r="B8">
-        <v>12436</v>
+        <v>12071</v>
       </c>
       <c r="C8">
-        <v>0</v>
+        <v>8971</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>5084</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>8216</v>
       </c>
       <c r="F8">
-        <v>0</v>
+        <v>3780</v>
       </c>
       <c r="G8">
-        <v>5559</v>
+        <v>4411</v>
       </c>
       <c r="H8">
-        <v>12172</v>
+        <v>8655</v>
       </c>
       <c r="I8">
-        <v>11658</v>
+        <v>8984</v>
       </c>
       <c r="J8">
-        <v>18042</v>
+        <v>16838</v>
       </c>
       <c r="K8">
-        <v>12328</v>
+        <v>7231</v>
       </c>
       <c r="L8">
-        <v>6903</v>
+        <v>3683</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -880,37 +868,37 @@
         <v>19</v>
       </c>
       <c r="B9">
-        <v>41766</v>
+        <v>10086</v>
       </c>
       <c r="C9">
-        <v>0</v>
+        <v>7193</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>3796</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>6242</v>
       </c>
       <c r="F9">
-        <v>0</v>
+        <v>2784</v>
       </c>
       <c r="G9">
-        <v>18311</v>
+        <v>3468</v>
       </c>
       <c r="H9">
-        <v>36641</v>
+        <v>6709</v>
       </c>
       <c r="I9">
-        <v>34464</v>
+        <v>7331</v>
       </c>
       <c r="J9">
-        <v>58893</v>
+        <v>13672</v>
       </c>
       <c r="K9">
-        <v>32025</v>
+        <v>5723</v>
       </c>
       <c r="L9">
-        <v>15570</v>
+        <v>3048</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -918,37 +906,37 @@
         <v>20</v>
       </c>
       <c r="B10">
-        <v>27756</v>
+        <v>12982</v>
       </c>
       <c r="C10">
-        <v>0</v>
+        <v>8623</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>4239</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>6674</v>
       </c>
       <c r="F10">
-        <v>0</v>
+        <v>3210</v>
       </c>
       <c r="G10">
-        <v>11002</v>
+        <v>4076</v>
       </c>
       <c r="H10">
-        <v>22453</v>
+        <v>8475</v>
       </c>
       <c r="I10">
-        <v>23742</v>
+        <v>8614</v>
       </c>
       <c r="J10">
-        <v>43091</v>
+        <v>16432</v>
       </c>
       <c r="K10">
-        <v>22493</v>
+        <v>6725</v>
       </c>
       <c r="L10">
-        <v>10703</v>
+        <v>3865</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -956,37 +944,37 @@
         <v>21</v>
       </c>
       <c r="B11">
-        <v>15999</v>
+        <v>5767</v>
       </c>
       <c r="C11">
-        <v>0</v>
+        <v>3738</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>1427</v>
       </c>
       <c r="E11">
-        <v>0</v>
+        <v>2479</v>
       </c>
       <c r="F11">
-        <v>0</v>
+        <v>1315</v>
       </c>
       <c r="G11">
-        <v>5484</v>
+        <v>1531</v>
       </c>
       <c r="H11">
-        <v>12086</v>
+        <v>3455</v>
       </c>
       <c r="I11">
-        <v>12262</v>
+        <v>3752</v>
       </c>
       <c r="J11">
-        <v>22427</v>
+        <v>6522</v>
       </c>
       <c r="K11">
-        <v>11271</v>
+        <v>2513</v>
       </c>
       <c r="L11">
-        <v>5764</v>
+        <v>1528</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -994,37 +982,37 @@
         <v>22</v>
       </c>
       <c r="B12">
-        <v>7051</v>
+        <v>3890</v>
       </c>
       <c r="C12">
-        <v>0</v>
+        <v>2197</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>1039</v>
       </c>
       <c r="E12">
-        <v>0</v>
+        <v>1353</v>
       </c>
       <c r="F12">
-        <v>0</v>
+        <v>1178</v>
       </c>
       <c r="G12">
-        <v>2088</v>
+        <v>1099</v>
       </c>
       <c r="H12">
-        <v>4947</v>
+        <v>1734</v>
       </c>
       <c r="I12">
-        <v>5170</v>
+        <v>1221</v>
       </c>
       <c r="J12">
-        <v>8838</v>
+        <v>1857</v>
       </c>
       <c r="K12">
-        <v>4288</v>
+        <v>1182</v>
       </c>
       <c r="L12">
-        <v>2303</v>
+        <v>640</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1032,74 +1020,36 @@
         <v>23</v>
       </c>
       <c r="B13">
-        <v>5725</v>
+        <v>9</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E13">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="F13">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="G13">
-        <v>1811</v>
+        <v>45</v>
       </c>
       <c r="H13">
-        <v>3113</v>
+        <v>21</v>
       </c>
       <c r="I13">
-        <v>2425</v>
+        <v>4</v>
       </c>
       <c r="J13">
-        <v>3714</v>
+        <v>3</v>
       </c>
       <c r="K13">
-        <v>3049</v>
+        <v>1</v>
       </c>
       <c r="L13">
-        <v>1643</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="A14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14">
-        <v>10</v>
-      </c>
-      <c r="C14">
-        <v>247662</v>
-      </c>
-      <c r="D14">
-        <v>118779</v>
-      </c>
-      <c r="E14">
-        <v>178147</v>
-      </c>
-      <c r="F14">
-        <v>102496</v>
-      </c>
-      <c r="G14">
-        <v>52</v>
-      </c>
-      <c r="H14">
-        <v>28</v>
-      </c>
-      <c r="I14">
-        <v>4</v>
-      </c>
-      <c r="J14">
-        <v>3</v>
-      </c>
-      <c r="K14">
-        <v>2</v>
-      </c>
-      <c r="L14">
         <v>0</v>
       </c>
     </row>
@@ -1110,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1">
@@ -1153,13 +1103,13 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2">
-        <v>89546</v>
+        <v>160273</v>
       </c>
       <c r="C2">
-        <v>166345</v>
+        <v>166367</v>
       </c>
       <c r="D2">
         <v>74562</v>
@@ -1174,7 +1124,7 @@
         <v>69195</v>
       </c>
       <c r="H2">
-        <v>148605</v>
+        <v>148607</v>
       </c>
       <c r="I2">
         <v>130196</v>
@@ -1186,68 +1136,68 @@
         <v>110477</v>
       </c>
       <c r="L2">
-        <v>56161</v>
+        <v>56651</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>41356</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>21633</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>13530</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>28218</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>30025</v>
       </c>
       <c r="G3">
-        <v>0</v>
+        <v>18136</v>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>26069</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>27817</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>31991</v>
       </c>
       <c r="K3">
-        <v>0</v>
+        <v>16173</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>10862</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B4">
-        <v>32131</v>
+        <v>37473</v>
       </c>
       <c r="C4">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4">
         <v>0</v>
       </c>
       <c r="G4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -1259,7 +1209,7 @@
         <v>0</v>
       </c>
       <c r="K4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L4">
         <v>0</v>
@@ -1267,13 +1217,13 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B5">
-        <v>70727</v>
+        <v>0</v>
       </c>
       <c r="C5">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1288,171 +1238,57 @@
         <v>0</v>
       </c>
       <c r="H5">
-        <v>2</v>
+        <v>74</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>385</v>
       </c>
       <c r="J5">
         <v>0</v>
       </c>
       <c r="K5">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="L5">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B6">
-        <v>45368</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>59634</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>30687</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>46348</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>28498</v>
+        <v>0</v>
       </c>
       <c r="G6">
-        <v>41659</v>
+        <v>0</v>
       </c>
       <c r="H6">
-        <v>99579</v>
+        <v>0</v>
       </c>
       <c r="I6">
-        <v>108044</v>
+        <v>0</v>
       </c>
       <c r="J6">
-        <v>162176</v>
+        <v>0</v>
       </c>
       <c r="K6">
-        <v>127054</v>
+        <v>0</v>
       </c>
       <c r="L6">
-        <v>64684</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7">
-        <v>41356</v>
-      </c>
-      <c r="C7">
-        <v>21633</v>
-      </c>
-      <c r="D7">
-        <v>13530</v>
-      </c>
-      <c r="E7">
-        <v>28218</v>
-      </c>
-      <c r="F7">
-        <v>30025</v>
-      </c>
-      <c r="G7">
-        <v>18136</v>
-      </c>
-      <c r="H7">
-        <v>26069</v>
-      </c>
-      <c r="I7">
-        <v>27817</v>
-      </c>
-      <c r="J7">
-        <v>31991</v>
-      </c>
-      <c r="K7">
-        <v>16173</v>
-      </c>
-      <c r="L7">
-        <v>10912</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12">
-      <c r="A8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8">
-        <v>37473</v>
-      </c>
-      <c r="C8">
-        <v>16</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <v>1</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>0</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>74</v>
-      </c>
-      <c r="I9">
-        <v>385</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>48</v>
-      </c>
-      <c r="L9">
-        <v>73</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1505,86 +1341,86 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B2">
-        <v>184260</v>
+        <v>128650</v>
       </c>
       <c r="C2">
-        <v>146798</v>
+        <v>113121</v>
       </c>
       <c r="D2">
-        <v>62163</v>
+        <v>50271</v>
       </c>
       <c r="E2">
-        <v>92393</v>
+        <v>69901</v>
       </c>
       <c r="F2">
-        <v>32937</v>
+        <v>22710</v>
       </c>
       <c r="G2">
-        <v>55950</v>
+        <v>37563</v>
       </c>
       <c r="H2">
-        <v>137526</v>
+        <v>85353</v>
       </c>
       <c r="I2">
-        <v>122048</v>
+        <v>72471</v>
       </c>
       <c r="J2">
-        <v>175841</v>
+        <v>124192</v>
       </c>
       <c r="K2">
-        <v>86689</v>
+        <v>44766</v>
       </c>
       <c r="L2">
-        <v>38521</v>
+        <v>22584</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B3">
-        <v>3741</v>
+        <v>3644</v>
       </c>
       <c r="C3">
-        <v>4493</v>
+        <v>4415</v>
       </c>
       <c r="D3">
-        <v>2446</v>
+        <v>2413</v>
       </c>
       <c r="E3">
-        <v>3632</v>
+        <v>3523</v>
       </c>
       <c r="F3">
-        <v>2010</v>
+        <v>1972</v>
       </c>
       <c r="G3">
-        <v>1419</v>
+        <v>1353</v>
       </c>
       <c r="H3">
-        <v>1909</v>
+        <v>1826</v>
       </c>
       <c r="I3">
-        <v>3743</v>
+        <v>3658</v>
       </c>
       <c r="J3">
-        <v>6062</v>
+        <v>5962</v>
       </c>
       <c r="K3">
-        <v>3976</v>
+        <v>3907</v>
       </c>
       <c r="L3">
-        <v>1800</v>
+        <v>1625</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4">
-        <v>76706</v>
+        <v>76442</v>
       </c>
       <c r="C4">
         <v>20469</v>
@@ -1614,50 +1450,50 @@
         <v>13664</v>
       </c>
       <c r="L4">
-        <v>9822</v>
+        <v>9798</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="B5">
-        <v>51895</v>
+        <v>30367</v>
       </c>
       <c r="C5">
-        <v>75902</v>
+        <v>50011</v>
       </c>
       <c r="D5">
-        <v>41490</v>
+        <v>22728</v>
       </c>
       <c r="E5">
-        <v>54956</v>
+        <v>31209</v>
       </c>
       <c r="F5">
-        <v>38618</v>
+        <v>20385</v>
       </c>
       <c r="G5">
-        <v>54100</v>
+        <v>30894</v>
       </c>
       <c r="H5">
-        <v>109427</v>
+        <v>62112</v>
       </c>
       <c r="I5">
-        <v>114584</v>
+        <v>56231</v>
       </c>
       <c r="J5">
-        <v>215193</v>
+        <v>104853</v>
       </c>
       <c r="K5">
-        <v>149357</v>
+        <v>64312</v>
       </c>
       <c r="L5">
-        <v>81613</v>
+        <v>33510</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -1678,19 +1514,19 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="I6">
-        <v>308</v>
+        <v>279</v>
       </c>
       <c r="J6">
-        <v>131</v>
+        <v>44</v>
       </c>
       <c r="K6">
-        <v>67</v>
+        <v>50</v>
       </c>
       <c r="L6">
-        <v>74</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1743,168 +1579,168 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B2">
-        <v>213552</v>
+        <v>150081</v>
       </c>
       <c r="C2">
-        <v>210831</v>
+        <v>157725</v>
       </c>
       <c r="D2">
-        <v>91218</v>
+        <v>66974</v>
       </c>
       <c r="E2">
-        <v>117093</v>
+        <v>82459</v>
       </c>
       <c r="F2">
-        <v>62752</v>
+        <v>39533</v>
       </c>
       <c r="G2">
-        <v>91291</v>
+        <v>58901</v>
       </c>
       <c r="H2">
-        <v>225474</v>
+        <v>140543</v>
       </c>
       <c r="I2">
-        <v>200669</v>
+        <v>120021</v>
       </c>
       <c r="J2">
-        <v>347598</v>
+        <v>219124</v>
       </c>
       <c r="K2">
-        <v>210610</v>
+        <v>102237</v>
       </c>
       <c r="L2">
-        <v>101011</v>
+        <v>50195</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B3">
-        <v>10481</v>
+        <v>4252</v>
       </c>
       <c r="C3">
-        <v>4884</v>
+        <v>3102</v>
       </c>
       <c r="D3">
-        <v>8395</v>
+        <v>4662</v>
       </c>
       <c r="E3">
-        <v>19556</v>
+        <v>13006</v>
       </c>
       <c r="F3">
-        <v>5289</v>
+        <v>2384</v>
       </c>
       <c r="G3">
-        <v>13553</v>
+        <v>7800</v>
       </c>
       <c r="H3">
-        <v>9056</v>
+        <v>3532</v>
       </c>
       <c r="I3">
-        <v>22151</v>
+        <v>3999</v>
       </c>
       <c r="J3">
-        <v>24564</v>
+        <v>3272</v>
       </c>
       <c r="K3">
-        <v>12670</v>
+        <v>3658</v>
       </c>
       <c r="L3">
-        <v>13597</v>
+        <v>4458</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4">
-        <v>91767</v>
+        <v>84280</v>
       </c>
       <c r="C4">
-        <v>31257</v>
+        <v>26842</v>
       </c>
       <c r="D4">
-        <v>18724</v>
+        <v>16329</v>
       </c>
       <c r="E4">
-        <v>41060</v>
+        <v>36193</v>
       </c>
       <c r="F4">
-        <v>34238</v>
+        <v>32006</v>
       </c>
       <c r="G4">
-        <v>23966</v>
+        <v>20581</v>
       </c>
       <c r="H4">
-        <v>39194</v>
+        <v>30443</v>
       </c>
       <c r="I4">
-        <v>41842</v>
+        <v>33796</v>
       </c>
       <c r="J4">
-        <v>52624</v>
+        <v>41174</v>
       </c>
       <c r="K4">
-        <v>29586</v>
+        <v>20516</v>
       </c>
       <c r="L4">
-        <v>16807</v>
+        <v>12764</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5">
+        <v>91</v>
+      </c>
+      <c r="C5">
         <v>37</v>
       </c>
-      <c r="B5">
-        <v>101</v>
-      </c>
-      <c r="C5">
-        <v>44</v>
-      </c>
       <c r="D5">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E5">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="F5">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G5">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H5">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I5">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="J5">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="K5">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="L5">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B6">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="C6">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D6">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E6">
         <v>101</v>
@@ -1922,56 +1758,56 @@
         <v>124</v>
       </c>
       <c r="J6">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K6">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="L6">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B7">
-        <v>369</v>
+        <v>71</v>
       </c>
       <c r="C7">
-        <v>383</v>
+        <v>49</v>
       </c>
       <c r="D7">
-        <v>325</v>
+        <v>24</v>
       </c>
       <c r="E7">
-        <v>301</v>
+        <v>16</v>
       </c>
       <c r="F7">
-        <v>166</v>
+        <v>26</v>
       </c>
       <c r="G7">
-        <v>153</v>
+        <v>23</v>
       </c>
       <c r="H7">
-        <v>309</v>
+        <v>36</v>
       </c>
       <c r="I7">
-        <v>372</v>
+        <v>57</v>
       </c>
       <c r="J7">
-        <v>653</v>
+        <v>74</v>
       </c>
       <c r="K7">
-        <v>503</v>
+        <v>67</v>
       </c>
       <c r="L7">
-        <v>199</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -1992,19 +1828,19 @@
         <v>0</v>
       </c>
       <c r="H8">
-        <v>166</v>
+        <v>70</v>
       </c>
       <c r="I8">
-        <v>1238</v>
+        <v>370</v>
       </c>
       <c r="J8">
-        <v>459</v>
+        <v>93</v>
       </c>
       <c r="K8">
-        <v>214</v>
+        <v>61</v>
       </c>
       <c r="L8">
-        <v>128</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -2057,1028 +1893,1028 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B2">
-        <v>1112</v>
+        <v>250</v>
       </c>
       <c r="C2">
-        <v>363</v>
+        <v>111</v>
       </c>
       <c r="D2">
-        <v>640</v>
+        <v>288</v>
       </c>
       <c r="E2">
-        <v>151</v>
+        <v>68</v>
       </c>
       <c r="F2">
-        <v>275</v>
+        <v>57</v>
       </c>
       <c r="G2">
-        <v>666</v>
+        <v>250</v>
       </c>
       <c r="H2">
-        <v>203</v>
+        <v>62</v>
       </c>
       <c r="I2">
-        <v>304</v>
+        <v>61</v>
       </c>
       <c r="J2">
-        <v>848</v>
+        <v>273</v>
       </c>
       <c r="K2">
-        <v>1387</v>
+        <v>171</v>
       </c>
       <c r="L2">
-        <v>342</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B3">
-        <v>19901</v>
+        <v>16386</v>
       </c>
       <c r="C3">
-        <v>666</v>
+        <v>488</v>
       </c>
       <c r="D3">
-        <v>424</v>
+        <v>207</v>
       </c>
       <c r="E3">
-        <v>2475</v>
+        <v>1754</v>
       </c>
       <c r="F3">
-        <v>291</v>
+        <v>171</v>
       </c>
       <c r="G3">
-        <v>824</v>
+        <v>601</v>
       </c>
       <c r="H3">
-        <v>12255</v>
+        <v>11173</v>
       </c>
       <c r="I3">
-        <v>1044</v>
+        <v>873</v>
       </c>
       <c r="J3">
-        <v>676</v>
+        <v>422</v>
       </c>
       <c r="K3">
-        <v>4747</v>
+        <v>3965</v>
       </c>
       <c r="L3">
-        <v>3471</v>
+        <v>3086</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B4">
-        <v>1180</v>
+        <v>258</v>
       </c>
       <c r="C4">
-        <v>660</v>
+        <v>226</v>
       </c>
       <c r="D4">
-        <v>620</v>
+        <v>193</v>
       </c>
       <c r="E4">
-        <v>191</v>
+        <v>30</v>
       </c>
       <c r="F4">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="G4">
-        <v>203</v>
+        <v>86</v>
       </c>
       <c r="H4">
-        <v>170</v>
+        <v>34</v>
       </c>
       <c r="I4">
-        <v>135</v>
+        <v>48</v>
       </c>
       <c r="J4">
-        <v>853</v>
+        <v>299</v>
       </c>
       <c r="K4">
-        <v>254</v>
+        <v>73</v>
       </c>
       <c r="L4">
-        <v>144</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B5">
-        <v>1115</v>
+        <v>444</v>
       </c>
       <c r="C5">
-        <v>601</v>
+        <v>249</v>
       </c>
       <c r="D5">
-        <v>205</v>
+        <v>71</v>
       </c>
       <c r="E5">
-        <v>206</v>
+        <v>88</v>
       </c>
       <c r="F5">
-        <v>124</v>
+        <v>34</v>
       </c>
       <c r="G5">
-        <v>370</v>
+        <v>163</v>
       </c>
       <c r="H5">
-        <v>471</v>
+        <v>165</v>
       </c>
       <c r="I5">
-        <v>582</v>
+        <v>241</v>
       </c>
       <c r="J5">
-        <v>482</v>
+        <v>95</v>
       </c>
       <c r="K5">
-        <v>489</v>
+        <v>181</v>
       </c>
       <c r="L5">
-        <v>246</v>
+        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B6">
-        <v>56170</v>
+        <v>52132</v>
       </c>
       <c r="C6">
-        <v>11550</v>
+        <v>9378</v>
       </c>
       <c r="D6">
-        <v>4547</v>
+        <v>3807</v>
       </c>
       <c r="E6">
-        <v>13180</v>
+        <v>11060</v>
       </c>
       <c r="F6">
-        <v>47109</v>
+        <v>41008</v>
       </c>
       <c r="G6">
-        <v>17911</v>
+        <v>14354</v>
       </c>
       <c r="H6">
-        <v>25090</v>
+        <v>18727</v>
       </c>
       <c r="I6">
-        <v>23186</v>
+        <v>15573</v>
       </c>
       <c r="J6">
-        <v>28134</v>
+        <v>16749</v>
       </c>
       <c r="K6">
-        <v>4740</v>
+        <v>2564</v>
       </c>
       <c r="L6">
-        <v>12895</v>
+        <v>10740</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B7">
-        <v>50304</v>
+        <v>38355</v>
       </c>
       <c r="C7">
-        <v>140406</v>
+        <v>114711</v>
       </c>
       <c r="D7">
-        <v>5612</v>
+        <v>1617</v>
       </c>
       <c r="E7">
-        <v>5772</v>
+        <v>1284</v>
       </c>
       <c r="F7">
-        <v>3760</v>
+        <v>1089</v>
       </c>
       <c r="G7">
-        <v>5350</v>
+        <v>1491</v>
       </c>
       <c r="H7">
-        <v>80295</v>
+        <v>52067</v>
       </c>
       <c r="I7">
-        <v>9398</v>
+        <v>2111</v>
       </c>
       <c r="J7">
-        <v>9802</v>
+        <v>1074</v>
       </c>
       <c r="K7">
-        <v>6020</v>
+        <v>853</v>
       </c>
       <c r="L7">
-        <v>6632</v>
+        <v>535</v>
       </c>
     </row>
     <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B8">
-        <v>1094</v>
+        <v>438</v>
       </c>
       <c r="C8">
-        <v>448</v>
+        <v>145</v>
       </c>
       <c r="D8">
-        <v>211</v>
+        <v>71</v>
       </c>
       <c r="E8">
-        <v>482</v>
+        <v>218</v>
       </c>
       <c r="F8">
-        <v>1569</v>
+        <v>146</v>
       </c>
       <c r="G8">
-        <v>334</v>
+        <v>235</v>
       </c>
       <c r="H8">
-        <v>1021</v>
+        <v>797</v>
       </c>
       <c r="I8">
-        <v>1173</v>
+        <v>820</v>
       </c>
       <c r="J8">
-        <v>1363</v>
+        <v>442</v>
       </c>
       <c r="K8">
-        <v>417</v>
+        <v>285</v>
       </c>
       <c r="L8">
-        <v>492</v>
+        <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B9">
-        <v>562</v>
+        <v>198</v>
       </c>
       <c r="C9">
-        <v>1693</v>
+        <v>838</v>
       </c>
       <c r="D9">
-        <v>1500</v>
+        <v>659</v>
       </c>
       <c r="E9">
-        <v>3400</v>
+        <v>1902</v>
       </c>
       <c r="F9">
-        <v>4883</v>
+        <v>4569</v>
       </c>
       <c r="G9">
         <v>0</v>
       </c>
       <c r="H9">
-        <v>3091</v>
+        <v>1163</v>
       </c>
       <c r="I9">
-        <v>18249</v>
+        <v>5321</v>
       </c>
       <c r="J9">
-        <v>22983</v>
+        <v>12715</v>
       </c>
       <c r="K9">
-        <v>6029</v>
+        <v>2353</v>
       </c>
       <c r="L9">
-        <v>975</v>
+        <v>161</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B10">
-        <v>550</v>
+        <v>82</v>
       </c>
       <c r="C10">
-        <v>662</v>
+        <v>179</v>
       </c>
       <c r="D10">
-        <v>522</v>
+        <v>179</v>
       </c>
       <c r="E10">
-        <v>346</v>
+        <v>104</v>
       </c>
       <c r="F10">
-        <v>182</v>
+        <v>51</v>
       </c>
       <c r="G10">
-        <v>1042</v>
+        <v>757</v>
       </c>
       <c r="H10">
-        <v>6015</v>
+        <v>4258</v>
       </c>
       <c r="I10">
-        <v>3999</v>
+        <v>2616</v>
       </c>
       <c r="J10">
-        <v>14456</v>
+        <v>10941</v>
       </c>
       <c r="K10">
-        <v>3633</v>
+        <v>2411</v>
       </c>
       <c r="L10">
-        <v>13286</v>
+        <v>11540</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B11">
-        <v>14677</v>
+        <v>12727</v>
       </c>
       <c r="C11">
-        <v>7971</v>
+        <v>6434</v>
       </c>
       <c r="D11">
-        <v>952</v>
+        <v>701</v>
       </c>
       <c r="E11">
-        <v>976</v>
+        <v>748</v>
       </c>
       <c r="F11">
-        <v>250</v>
+        <v>209</v>
       </c>
       <c r="G11">
-        <v>274</v>
+        <v>246</v>
       </c>
       <c r="H11">
-        <v>3426</v>
+        <v>2198</v>
       </c>
       <c r="I11">
-        <v>4270</v>
+        <v>2847</v>
       </c>
       <c r="J11">
-        <v>2617</v>
+        <v>980</v>
       </c>
       <c r="K11">
-        <v>1576</v>
+        <v>570</v>
       </c>
       <c r="L11">
-        <v>1803</v>
+        <v>458</v>
       </c>
     </row>
     <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B12">
-        <v>1511</v>
+        <v>449</v>
       </c>
       <c r="C12">
-        <v>3929</v>
+        <v>3511</v>
       </c>
       <c r="D12">
-        <v>14360</v>
+        <v>13542</v>
       </c>
       <c r="E12">
-        <v>889</v>
+        <v>510</v>
       </c>
       <c r="F12">
-        <v>804</v>
+        <v>345</v>
       </c>
       <c r="G12">
-        <v>345</v>
+        <v>193</v>
       </c>
       <c r="H12">
-        <v>466</v>
+        <v>219</v>
       </c>
       <c r="I12">
-        <v>711</v>
+        <v>337</v>
       </c>
       <c r="J12">
-        <v>25693</v>
+        <v>21782</v>
       </c>
       <c r="K12">
-        <v>66556</v>
+        <v>49289</v>
       </c>
       <c r="L12">
-        <v>2588</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B13">
-        <v>421</v>
+        <v>98</v>
       </c>
       <c r="C13">
-        <v>568</v>
+        <v>156</v>
       </c>
       <c r="D13">
-        <v>821</v>
+        <v>273</v>
       </c>
       <c r="E13">
-        <v>698</v>
+        <v>167</v>
       </c>
       <c r="F13">
-        <v>426</v>
+        <v>191</v>
       </c>
       <c r="G13">
-        <v>525</v>
+        <v>170</v>
       </c>
       <c r="H13">
-        <v>4345</v>
+        <v>592</v>
       </c>
       <c r="I13">
-        <v>15656</v>
+        <v>2702</v>
       </c>
       <c r="J13">
-        <v>33793</v>
+        <v>2453</v>
       </c>
       <c r="K13">
-        <v>50493</v>
+        <v>12401</v>
       </c>
       <c r="L13">
-        <v>35313</v>
+        <v>12233</v>
       </c>
     </row>
     <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B14">
-        <v>2421</v>
+        <v>658</v>
       </c>
       <c r="C14">
-        <v>20853</v>
+        <v>16439</v>
       </c>
       <c r="D14">
-        <v>13461</v>
+        <v>11849</v>
       </c>
       <c r="E14">
-        <v>5050</v>
+        <v>2679</v>
       </c>
       <c r="F14">
-        <v>5126</v>
+        <v>3380</v>
       </c>
       <c r="G14">
-        <v>7721</v>
+        <v>5386</v>
       </c>
       <c r="H14">
-        <v>17048</v>
+        <v>12277</v>
       </c>
       <c r="I14">
-        <v>130426</v>
+        <v>100693</v>
       </c>
       <c r="J14">
-        <v>196968</v>
+        <v>166731</v>
       </c>
       <c r="K14">
-        <v>27654</v>
+        <v>20127</v>
       </c>
       <c r="L14">
-        <v>21642</v>
+        <v>15882</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B15">
-        <v>4614</v>
+        <v>3448</v>
       </c>
       <c r="C15">
-        <v>11867</v>
+        <v>8821</v>
       </c>
       <c r="D15">
-        <v>12350</v>
+        <v>7840</v>
       </c>
       <c r="E15">
-        <v>6261</v>
+        <v>3494</v>
       </c>
       <c r="F15">
-        <v>1968</v>
+        <v>405</v>
       </c>
       <c r="G15">
-        <v>946</v>
+        <v>182</v>
       </c>
       <c r="H15">
-        <v>1583</v>
+        <v>263</v>
       </c>
       <c r="I15">
-        <v>2375</v>
+        <v>469</v>
       </c>
       <c r="J15">
-        <v>6990</v>
+        <v>965</v>
       </c>
       <c r="K15">
-        <v>3228</v>
+        <v>638</v>
       </c>
       <c r="L15">
-        <v>1401</v>
+        <v>314</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B16">
-        <v>20855</v>
+        <v>18859</v>
       </c>
       <c r="C16">
-        <v>1992</v>
+        <v>1806</v>
       </c>
       <c r="D16">
-        <v>1488</v>
+        <v>1059</v>
       </c>
       <c r="E16">
-        <v>2059</v>
+        <v>1662</v>
       </c>
       <c r="F16">
-        <v>2432</v>
+        <v>1975</v>
       </c>
       <c r="G16">
-        <v>12345</v>
+        <v>10710</v>
       </c>
       <c r="H16">
-        <v>24342</v>
+        <v>18876</v>
       </c>
       <c r="I16">
-        <v>2201</v>
+        <v>1419</v>
       </c>
       <c r="J16">
-        <v>5676</v>
+        <v>1693</v>
       </c>
       <c r="K16">
-        <v>3721</v>
+        <v>551</v>
       </c>
       <c r="L16">
-        <v>1888</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B17">
-        <v>2714</v>
+        <v>467</v>
       </c>
       <c r="C17">
-        <v>828</v>
+        <v>168</v>
       </c>
       <c r="D17">
-        <v>645</v>
+        <v>122</v>
       </c>
       <c r="E17">
-        <v>837</v>
+        <v>223</v>
       </c>
       <c r="F17">
-        <v>706</v>
+        <v>414</v>
       </c>
       <c r="G17">
-        <v>366</v>
+        <v>188</v>
       </c>
       <c r="H17">
-        <v>428</v>
+        <v>168</v>
       </c>
       <c r="I17">
-        <v>3862</v>
+        <v>1895</v>
       </c>
       <c r="J17">
-        <v>2066</v>
+        <v>800</v>
       </c>
       <c r="K17">
-        <v>11683</v>
+        <v>7109</v>
       </c>
       <c r="L17">
-        <v>1476</v>
+        <v>291</v>
       </c>
     </row>
     <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B18">
-        <v>63161</v>
+        <v>37169</v>
       </c>
       <c r="C18">
-        <v>5543</v>
+        <v>1990</v>
       </c>
       <c r="D18">
-        <v>3658</v>
+        <v>1224</v>
       </c>
       <c r="E18">
-        <v>8962</v>
+        <v>2614</v>
       </c>
       <c r="F18">
-        <v>8685</v>
+        <v>5454</v>
       </c>
       <c r="G18">
-        <v>36486</v>
+        <v>26442</v>
       </c>
       <c r="H18">
-        <v>35515</v>
+        <v>16381</v>
       </c>
       <c r="I18">
-        <v>7453</v>
+        <v>2548</v>
       </c>
       <c r="J18">
-        <v>15538</v>
+        <v>4350</v>
       </c>
       <c r="K18">
-        <v>7673</v>
+        <v>2533</v>
       </c>
       <c r="L18">
-        <v>7017</v>
+        <v>2136</v>
       </c>
     </row>
     <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B19">
-        <v>3082</v>
+        <v>2122</v>
       </c>
       <c r="C19">
-        <v>8190</v>
+        <v>6433</v>
       </c>
       <c r="D19">
-        <v>929</v>
+        <v>650</v>
       </c>
       <c r="E19">
-        <v>1226</v>
+        <v>887</v>
       </c>
       <c r="F19">
-        <v>295</v>
+        <v>193</v>
       </c>
       <c r="G19">
-        <v>480</v>
+        <v>255</v>
       </c>
       <c r="H19">
-        <v>12300</v>
+        <v>10786</v>
       </c>
       <c r="I19">
-        <v>5238</v>
+        <v>4403</v>
       </c>
       <c r="J19">
-        <v>1322</v>
+        <v>883</v>
       </c>
       <c r="K19">
-        <v>986</v>
+        <v>624</v>
       </c>
       <c r="L19">
-        <v>615</v>
+        <v>479</v>
       </c>
     </row>
     <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B20">
-        <v>27392</v>
+        <v>24562</v>
       </c>
       <c r="C20">
-        <v>2454</v>
+        <v>2121</v>
       </c>
       <c r="D20">
-        <v>3714</v>
+        <v>2221</v>
       </c>
       <c r="E20">
-        <v>15491</v>
+        <v>13649</v>
       </c>
       <c r="F20">
-        <v>7813</v>
+        <v>5457</v>
       </c>
       <c r="G20">
-        <v>5923</v>
+        <v>4672</v>
       </c>
       <c r="H20">
-        <v>19554</v>
+        <v>13792</v>
       </c>
       <c r="I20">
-        <v>3637</v>
+        <v>2278</v>
       </c>
       <c r="J20">
-        <v>6110</v>
+        <v>2899</v>
       </c>
       <c r="K20">
-        <v>4674</v>
+        <v>3041</v>
       </c>
       <c r="L20">
-        <v>1775</v>
+        <v>974</v>
       </c>
     </row>
     <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B21">
-        <v>664</v>
+        <v>126</v>
       </c>
       <c r="C21">
-        <v>407</v>
+        <v>75</v>
       </c>
       <c r="D21">
-        <v>295</v>
+        <v>54</v>
       </c>
       <c r="E21">
-        <v>343</v>
+        <v>76</v>
       </c>
       <c r="F21">
-        <v>266</v>
+        <v>46</v>
       </c>
       <c r="G21">
-        <v>673</v>
+        <v>313</v>
       </c>
       <c r="H21">
-        <v>756</v>
+        <v>234</v>
       </c>
       <c r="I21">
-        <v>578</v>
+        <v>188</v>
       </c>
       <c r="J21">
-        <v>912</v>
+        <v>340</v>
       </c>
       <c r="K21">
-        <v>1500</v>
+        <v>529</v>
       </c>
       <c r="L21">
-        <v>415</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B22">
-        <v>19652</v>
+        <v>17634</v>
       </c>
       <c r="C22">
-        <v>5959</v>
+        <v>4813</v>
       </c>
       <c r="D22">
-        <v>45405</v>
+        <v>40298</v>
       </c>
       <c r="E22">
-        <v>99390</v>
+        <v>86630</v>
       </c>
       <c r="F22">
-        <v>5923</v>
+        <v>4127</v>
       </c>
       <c r="G22">
-        <v>1165</v>
+        <v>548</v>
       </c>
       <c r="H22">
-        <v>1673</v>
+        <v>699</v>
       </c>
       <c r="I22">
-        <v>3416</v>
+        <v>1444</v>
       </c>
       <c r="J22">
-        <v>7138</v>
+        <v>4637</v>
       </c>
       <c r="K22">
-        <v>4261</v>
+        <v>1807</v>
       </c>
       <c r="L22">
-        <v>4644</v>
+        <v>2882</v>
       </c>
     </row>
     <row r="23" spans="1:12">
       <c r="A23" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23">
+        <v>476</v>
+      </c>
+      <c r="C23">
+        <v>216</v>
+      </c>
+      <c r="D23">
         <v>61</v>
       </c>
-      <c r="B23">
-        <v>1879</v>
-      </c>
-      <c r="C23">
-        <v>863</v>
-      </c>
-      <c r="D23">
-        <v>464</v>
-      </c>
       <c r="E23">
-        <v>576</v>
+        <v>107</v>
       </c>
       <c r="F23">
-        <v>1079</v>
+        <v>107</v>
       </c>
       <c r="G23">
-        <v>433</v>
+        <v>135</v>
       </c>
       <c r="H23">
-        <v>517</v>
+        <v>141</v>
       </c>
       <c r="I23">
-        <v>984</v>
+        <v>58</v>
       </c>
       <c r="J23">
-        <v>2241</v>
+        <v>222</v>
       </c>
       <c r="K23">
-        <v>10365</v>
+        <v>4593</v>
       </c>
       <c r="L23">
-        <v>2500</v>
+        <v>1142</v>
       </c>
     </row>
     <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B24">
-        <v>296</v>
+        <v>31</v>
       </c>
       <c r="C24">
-        <v>6760</v>
+        <v>4015</v>
       </c>
       <c r="D24">
-        <v>508</v>
+        <v>42</v>
       </c>
       <c r="E24">
-        <v>510</v>
+        <v>40</v>
       </c>
       <c r="F24">
-        <v>155</v>
+        <v>10</v>
       </c>
       <c r="G24">
-        <v>341</v>
+        <v>52</v>
       </c>
       <c r="H24">
-        <v>442</v>
+        <v>101</v>
       </c>
       <c r="I24">
-        <v>503</v>
+        <v>26</v>
       </c>
       <c r="J24">
-        <v>738</v>
+        <v>40</v>
       </c>
       <c r="K24">
-        <v>312</v>
+        <v>48</v>
       </c>
       <c r="L24">
-        <v>136</v>
+        <v>31</v>
       </c>
     </row>
     <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B25">
-        <v>1014</v>
+        <v>174</v>
       </c>
       <c r="C25">
-        <v>427</v>
+        <v>56</v>
       </c>
       <c r="D25">
-        <v>403</v>
+        <v>55</v>
       </c>
       <c r="E25">
-        <v>703</v>
+        <v>117</v>
       </c>
       <c r="F25">
-        <v>668</v>
+        <v>98</v>
       </c>
       <c r="G25">
-        <v>530</v>
+        <v>114</v>
       </c>
       <c r="H25">
-        <v>850</v>
+        <v>163</v>
       </c>
       <c r="I25">
-        <v>944</v>
+        <v>223</v>
       </c>
       <c r="J25">
-        <v>1091</v>
+        <v>142</v>
       </c>
       <c r="K25">
-        <v>2999</v>
+        <v>857</v>
       </c>
       <c r="L25">
-        <v>674</v>
+        <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:12">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B26">
-        <v>7063</v>
+        <v>2080</v>
       </c>
       <c r="C26">
-        <v>4489</v>
+        <v>992</v>
       </c>
       <c r="D26">
-        <v>3561</v>
+        <v>701</v>
       </c>
       <c r="E26">
-        <v>5557</v>
+        <v>1203</v>
       </c>
       <c r="F26">
-        <v>2239</v>
+        <v>576</v>
       </c>
       <c r="G26">
-        <v>26810</v>
+        <v>16447</v>
       </c>
       <c r="H26">
-        <v>4950</v>
+        <v>1342</v>
       </c>
       <c r="I26">
-        <v>9959</v>
+        <v>3077</v>
       </c>
       <c r="J26">
-        <v>31333</v>
+        <v>10906</v>
       </c>
       <c r="K26">
-        <v>25438</v>
+        <v>8451</v>
       </c>
       <c r="L26">
-        <v>7540</v>
+        <v>2075</v>
       </c>
     </row>
     <row r="27" spans="1:12">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B27">
-        <v>11007</v>
+        <v>8827</v>
       </c>
       <c r="C27">
-        <v>802</v>
+        <v>497</v>
       </c>
       <c r="D27">
-        <v>95</v>
+        <v>42</v>
       </c>
       <c r="E27">
-        <v>714</v>
+        <v>293</v>
       </c>
       <c r="F27">
-        <v>4997</v>
+        <v>3822</v>
       </c>
       <c r="G27">
-        <v>5784</v>
+        <v>3067</v>
       </c>
       <c r="H27">
-        <v>8386</v>
+        <v>4003</v>
       </c>
       <c r="I27">
-        <v>4708</v>
+        <v>1565</v>
       </c>
       <c r="J27">
-        <v>2535</v>
+        <v>444</v>
       </c>
       <c r="K27">
-        <v>1236</v>
+        <v>195</v>
       </c>
       <c r="L27">
-        <v>940</v>
+        <v>338</v>
       </c>
     </row>
     <row r="28" spans="1:12">
       <c r="A28" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B28">
-        <v>2191</v>
+        <v>653</v>
       </c>
       <c r="C28">
-        <v>6711</v>
+        <v>3148</v>
       </c>
       <c r="D28">
-        <v>1389</v>
+        <v>266</v>
       </c>
       <c r="E28">
-        <v>1702</v>
+        <v>192</v>
       </c>
       <c r="F28">
-        <v>427</v>
+        <v>56</v>
       </c>
       <c r="G28">
-        <v>1144</v>
+        <v>275</v>
       </c>
       <c r="H28">
-        <v>9139</v>
+        <v>4070</v>
       </c>
       <c r="I28">
-        <v>11451</v>
+        <v>4562</v>
       </c>
       <c r="J28">
-        <v>3856</v>
+        <v>761</v>
       </c>
       <c r="K28">
-        <v>1682</v>
+        <v>480</v>
       </c>
       <c r="L28">
-        <v>980</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -3131,89 +2967,89 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B2">
-        <v>199388</v>
+        <v>150603</v>
       </c>
       <c r="C2">
-        <v>152113</v>
+        <v>116129</v>
       </c>
       <c r="D2">
-        <v>72444</v>
+        <v>54375</v>
       </c>
       <c r="E2">
-        <v>107761</v>
+        <v>80479</v>
       </c>
       <c r="F2">
-        <v>61125</v>
+        <v>44481</v>
       </c>
       <c r="G2">
-        <v>76717</v>
+        <v>52449</v>
       </c>
       <c r="H2">
-        <v>166195</v>
+        <v>107220</v>
       </c>
       <c r="I2">
-        <v>156668</v>
+        <v>94533</v>
       </c>
       <c r="J2">
-        <v>251700</v>
+        <v>157667</v>
       </c>
       <c r="K2">
-        <v>148482</v>
+        <v>75928</v>
       </c>
       <c r="L2">
-        <v>75596</v>
+        <v>39480</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B3">
-        <v>254</v>
+        <v>193</v>
       </c>
       <c r="C3">
-        <v>162</v>
+        <v>132</v>
       </c>
       <c r="D3">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="E3">
-        <v>405</v>
+        <v>334</v>
       </c>
       <c r="F3">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="G3">
-        <v>132</v>
+        <v>80</v>
       </c>
       <c r="H3">
-        <v>266</v>
+        <v>193</v>
       </c>
       <c r="I3">
-        <v>483</v>
+        <v>389</v>
       </c>
       <c r="J3">
-        <v>392</v>
+        <v>267</v>
       </c>
       <c r="K3">
-        <v>161</v>
+        <v>109</v>
       </c>
       <c r="L3">
-        <v>75</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4">
         <v>4</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <v>2</v>
@@ -3225,7 +3061,7 @@
         <v>0</v>
       </c>
       <c r="G4">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H4">
         <v>2</v>
@@ -3234,7 +3070,7 @@
         <v>0</v>
       </c>
       <c r="J4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -3245,40 +3081,40 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B5">
-        <v>116956</v>
+        <v>88303</v>
       </c>
       <c r="C5">
-        <v>95386</v>
+        <v>71755</v>
       </c>
       <c r="D5">
-        <v>46210</v>
+        <v>33610</v>
       </c>
       <c r="E5">
-        <v>69981</v>
+        <v>50986</v>
       </c>
       <c r="F5">
-        <v>41230</v>
+        <v>29400</v>
       </c>
       <c r="G5">
-        <v>52137</v>
+        <v>34799</v>
       </c>
       <c r="H5">
-        <v>107868</v>
+        <v>67336</v>
       </c>
       <c r="I5">
-        <v>109291</v>
+        <v>63476</v>
       </c>
       <c r="J5">
-        <v>174120</v>
+        <v>106103</v>
       </c>
       <c r="K5">
-        <v>105110</v>
+        <v>50662</v>
       </c>
       <c r="L5">
-        <v>56159</v>
+        <v>28027</v>
       </c>
     </row>
   </sheetData>

</xml_diff>